<commit_message>
fix: publish observed ST generator and grid MW masters with exact response diagram
</commit_message>
<xml_diff>
--- a/data/current_v8/masters/07_LOGIC_MASTER_CURRENT_V8_VERIFIED.xlsx
+++ b/data/current_v8/masters/07_LOGIC_MASTER_CURRENT_V8_VERIFIED.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Verification" sheetId="1" r:id="Rc426ec305328487a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Logic_Master_Current" sheetId="2" r:id="R23978f92cdce439d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Logic_Edges" sheetId="3" r:id="Re825307e4c374d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Group_View" sheetId="4" r:id="R6a4c0473b2f14522"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Source_Notes" sheetId="5" r:id="Re98c257c877c4741"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Logic_Master_Grouped" sheetId="6" r:id="R0bb7fb3940494bbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Input_Groups" sheetId="7" r:id="Rb71e77017c454af6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Tag_Identity_Policy" sheetId="8" r:id="Ra0c7f7bbcfc046f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Verification" sheetId="1" r:id="R501f8088b80f486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Logic_Master_Current" sheetId="2" r:id="Ra06c5124e7ae42db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Logic_Edges" sheetId="3" r:id="R812715d876e8427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Group_View" sheetId="4" r:id="R5d40695c9a544d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Source_Notes" sheetId="5" r:id="R45477515479642a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Logic_Master_Grouped" sheetId="6" r:id="Rc9c9a6284bf240e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Input_Groups" sheetId="7" r:id="R770d0c7509b14639"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Tag_Identity_Policy" sheetId="8" r:id="R53545d04a29f4ecf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -332,7 +332,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CurrentLogicMaster" displayName="CurrentLogicMaster" ref="A1:O54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CurrentLogicMaster" displayName="CurrentLogicMaster" ref="A1:O55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="rule_id"/>
     <x:tableColumn id="2" name="group"/>
@@ -652,10 +652,10 @@
         <x:v>Current logic rows</x:v>
       </x:c>
       <x:c r="B3" s="8" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C3" s="8" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
         <x:v>PASS</x:v>
@@ -663,44 +663,44 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="8" t="str">
-        <x:v>Unique source input nodes live</x:v>
+        <x:v>Unique source input nodes observed</x:v>
       </x:c>
       <x:c r="B4" s="8" t="n">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C4" s="8" t="n">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D4" s="8" t="str">
-        <x:v>PASS</x:v>
+        <x:v>IDENTITY_OBSERVED</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
-        <x:v>Rules with all inputs live</x:v>
+        <x:v>Rules with all inputs observed</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C5" s="8" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D5" s="8" t="str">
-        <x:v>PASS</x:v>
+        <x:v>IDENTITY_OBSERVED</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8" t="str">
-        <x:v>Unique vpp source/model outputs live</x:v>
+        <x:v>Unique vpp source/model outputs observed</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C6" s="8" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>PASS</x:v>
+        <x:v>IDENTITY_OBSERVED</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -761,16 +761,16 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
-        <x:v>Live Tag Master source nodes</x:v>
+        <x:v>Current Tag Master source nodes</x:v>
       </x:c>
       <x:c r="B11" s="8" t="n">
-        <x:v>603</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="C11" s="8" t="n">
-        <x:v>603</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="D11" s="8" t="str">
-        <x:v>PASS</x:v>
+        <x:v>IDENTITY_OBSERVED</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -789,16 +789,16 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
-        <x:v>Behavior evidence</x:v>
+        <x:v>ST power behavior evidence</x:v>
       </x:c>
       <x:c r="B13" s="8" t="str">
-        <x:v>Run #41 columns retained separately</x:v>
+        <x:v>282 closed-breaker observations</x:v>
       </x:c>
       <x:c r="C13" s="8" t="str">
-        <x:v>Identity/current-existence is determined by Run #54 live census</x:v>
+        <x:v>52ST open -&gt; 0 MW not behaviorally tested</x:v>
       </x:c>
       <x:c r="D13" s="8" t="str">
-        <x:v>INFO</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5695,6 +5695,96 @@
         <x:v>inputs=1 live=1; vpp_outputs=1 live=1; local_derived_outputs=0</x:v>
       </x:c>
     </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="8" t="str">
+        <x:v>RESP-ST-GRID-POWER</x:v>
+      </x:c>
+      <x:c r="B55" s="8" t="str">
+        <x:v>ST Protection</x:v>
+      </x:c>
+      <x:c r="C55" s="8" t="str">
+        <x:v>ST grid power response after 52ST opens</x:v>
+      </x:c>
+      <x:c r="D55" s="8" t="str">
+        <x:v>PHYSICAL_RESPONSE</x:v>
+      </x:c>
+      <x:c r="E55" s="8" t="str">
+        <x:v>vpp52STClosed | vppSTGeneratorPowerMW</x:v>
+      </x:c>
+      <x:c r="F55" s="8" t="str">
+        <x:v>if 52ST not closed then ST grid power = 0; otherwise ST grid power = ST generator power</x:v>
+      </x:c>
+      <x:c r="G55" s="8" t="str">
+        <x:v>immediate model relation</x:v>
+      </x:c>
+      <x:c r="H55" s="8" t="str">
+        <x:v>follows 52ST closed feedback</x:v>
+      </x:c>
+      <x:c r="I55" s="8" t="str">
+        <x:v>vppSTGridPowerMW</x:v>
+      </x:c>
+      <x:c r="J55" s="8" t="str">
+        <x:v>RAW_NODE</x:v>
+      </x:c>
+      <x:c r="K55" s="8" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="L55" s="8" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="M55" s="8" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="N55" s="8" t="str">
+        <x:v>Local PlantControlV2 exact equation and supplemental RAW observations; data/current_v8/st_power_evidence_20260924.json</x:v>
+      </x:c>
+      <x:c r="O55" s="8" t="str">
+        <x:v>PHYSICAL_RESPONSE, not a new trip cause or threshold. 52ST-closed branch observed; 52ST-open zero response remains UNTESTED.</x:v>
+      </x:c>
+      <x:c r="P55" s="8" t="str">
+        <x:v>IG-036</x:v>
+      </x:c>
+      <x:c r="Q55" s="8" t="str">
+        <x:v>vpp52STClosed | vppSTGeneratorPowerMW</x:v>
+      </x:c>
+      <x:c r="R55" s="8" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S55" s="8" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T55" s="8" t="str">
+        <x:v>NOT_IN_RUN41</x:v>
+      </x:c>
+      <x:c r="U55" s="8" t="str">
+        <x:v>RC_EVIDENCE_AVAILABLE</x:v>
+      </x:c>
+      <x:c r="V55" s="8" t="str"/>
+      <x:c r="W55" s="8" t="str">
+        <x:v>Added from current PlantControlV2 source and RAW session.</x:v>
+      </x:c>
+      <x:c r="X55" s="8" t="str">
+        <x:v>EXACT_RAW_OR_SOURCE_NODE</x:v>
+      </x:c>
+      <x:c r="Y55" s="8" t="str">
+        <x:v>EXACT_RAW_OR_SOURCE_NODE</x:v>
+      </x:c>
+      <x:c r="Z55" s="8" t="str">
+        <x:v>PASS_NO_INVENTED_INPUT_NODE</x:v>
+      </x:c>
+      <x:c r="AA55" s="8" t="str">
+        <x:v>PASS_CENSUS_AND_RAW_READBACK</x:v>
+      </x:c>
+      <x:c r="AB55" s="8" t="str">
+        <x:v>PASS_RAW_SESSION_READBACK</x:v>
+      </x:c>
+      <x:c r="AC55" s="8" t="str">
+        <x:v>SESSION_20260924_191347</x:v>
+      </x:c>
+      <x:c r="AD55" s="8" t="str">
+        <x:v>vpp52STClosed: Run 54 census; both ST MW signals: 282 current RAW observations. Native node IDs/types not captured; open-breaker behavior untested.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="K2:L54">
     <x:cfRule type="expression" dxfId="0" priority="1">
@@ -5703,7 +5793,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd51e32c0758648a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R376b40dc288a437e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8596,7 +8686,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R177e0ce52d6d469c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe90a4e888964810"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8904,7 +8994,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fe5213cc2a04ba7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e038d8cad5948a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13554,7 +13644,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5966b27f3c6b4cd5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc831f40a56ea45cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15277,7 +15367,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365d08ef284b487f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8931f43d55104c59"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>